<commit_message>
mock up 1 runnable
</commit_message>
<xml_diff>
--- a/XmlData/Datas/__beans__.xlsx
+++ b/XmlData/Datas/__beans__.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinya\Documents\unityProjects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7250B0E-E5F6-4127-B05C-12AC22B3E030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864D40C8-9A49-4C20-8428-5D8DEDF52AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23940" yWindow="-360" windowWidth="21600" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -101,9 +101,6 @@
     <t>WordChoice</t>
   </si>
   <si>
-    <t>(string#sep=,)</t>
-  </si>
-  <si>
     <t>Enum.CheeseWord</t>
   </si>
   <si>
@@ -114,13 +111,16 @@
   </si>
   <si>
     <t>词性</t>
+  </si>
+  <si>
+    <t>(list#sep=,),string</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,6 +164,11 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -205,7 +210,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -213,12 +218,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -538,15 +546,15 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
@@ -604,30 +612,30 @@
       </c>
     </row>
     <row r="4" spans="1:16">
-      <c r="B4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="4"/>
+      <c r="B4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="3"/>
       <c r="J4" t="s">
         <v>23</v>
       </c>
       <c r="L4" t="s">
-        <v>26</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
-      <c r="C5" s="4"/>
+    <row r="5" spans="1:16" ht="17.25">
+      <c r="C5" s="3"/>
       <c r="J5" t="s">
         <v>24</v>
       </c>
-      <c r="L5" t="s">
-        <v>25</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>28</v>
+      <c r="L5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update cheeseWord enum to cheeseWordData enum
</commit_message>
<xml_diff>
--- a/XmlData/Datas/__beans__.xlsx
+++ b/XmlData/Datas/__beans__.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinya\Documents\unityProjects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864D40C8-9A49-4C20-8428-5D8DEDF52AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E26AEE-8073-477B-9C0A-2C7BBFD1971D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23940" yWindow="-360" windowWidth="21600" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -101,9 +101,6 @@
     <t>WordChoice</t>
   </si>
   <si>
-    <t>Enum.CheeseWord</t>
-  </si>
-  <si>
     <t>WordContent</t>
   </si>
   <si>
@@ -114,6 +111,9 @@
   </si>
   <si>
     <t>(list#sep=,),string</t>
+  </si>
+  <si>
+    <t>Enum.CheeseWordData</t>
   </si>
 </sst>
 </file>
@@ -223,11 +223,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -546,15 +546,15 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
@@ -613,17 +613,17 @@
     </row>
     <row r="4" spans="1:16">
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4" s="3"/>
       <c r="J4" t="s">
         <v>23</v>
       </c>
       <c r="L4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="17.25">
@@ -631,11 +631,11 @@
       <c r="J5" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="5" t="s">
-        <v>29</v>
+      <c r="L5" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>